<commit_message>
Epic 3 S6 (E3-06.4 DONE): guard JSON parse in vision extractors (crash-hardening)
S6/S7 completeness audit finding: ai_extract_document (ingestion.py) and
ai_extract_ledger_file (ledger.py) called _extract_json(resp) UNGUARDED, so a
malformed OCR response raised and crashed the ingest/ledger flow -- while their
siblings ai_map_spreadsheet (E3-06.3) and ai_extract (E3-02.1) were already
hardened. Both now try/except -> degrade to {} and record telemetry parse_ok=False,
so a bad OCR parse is observable instead of fatal.

Verified: raw _extract_json raises JSONDecodeError on non-JSON; both extractors now
catch it. Exit gate + fingerprint (260) hold.

Trackers side-by-side: Epic 3 Sprint 6 -> 4/4; Master Epic 3 -> 14/37. Dashboard regenerated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic3_AI_Foundation.xlsx
+++ b/docs/DecisionOS_Epic3_AI_Foundation.xlsx
@@ -1149,10 +1149,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1313,7 +1313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3544,6 +3544,66 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>E3-06.4</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>services/ingestion.py + routers/ledger.py</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>6</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Document AI</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Vision extractors: guard JSON parse (crash-hardening)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Audit finding (S6/S7 completeness review): ai_extract_document + ai_extract_ledger_file called _extract_json(resp) UNGUARDED, so a malformed OCR response RAISED and crashed the ingest/ledger flow (ai_map_spreadsheet + ai_extract were already guarded). Both now try/except -&gt; degrade to {} and set telemetry parse_ok=False for observability. Fingerprint 260.</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>E3-01.3</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Found + fixed 2026-08-25 during the founder-requested S6/S7 completeness check. Same class as the ai_map_spreadsheet guard (E3-06.3). Verified: raw _extract_json raises JSONDecodeError on garbage; both extractors now catch it.</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Epic 3 S6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(tracker): capture S6/S7 audit findings as backlog (E3-06.5/.6/.7)
The founder-requested completeness audit surfaced three open gaps beyond the fixed
crash bug (E3-06.4). Captured so they aren't lost:
- E3-06.5 (P1) extend duplicate detection to payments + expenses/assets (invoices
  only today -- same double-entry money risk).
- E3-06.6 (P2) confidence calibration + review-routing for document/vision
  extraction (extend the E3-02.2 pattern to ai_extract_document).
- E3-06.7 (P3) tolerant amount/currency parsing (lakh/crore/₹/commas) for the
  India market.

Epic 3 -> 14/40; Sprint 6 -> 4/7 (E3-06.1 deferred, .2/.3/.4 done, .5/.6/.7 backlog).
Dashboard regenerated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic3_AI_Foundation.xlsx
+++ b/docs/DecisionOS_Epic3_AI_Foundation.xlsx
@@ -1152,16 +1152,16 @@
         <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>57%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Done (1 deferred: testing)</t>
+          <t>In progress (1 deferred: testing)</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -1313,7 +1313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3604,6 +3604,182 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>E3-06.5</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>services/ingestion.py (dedup)</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>6</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Document AI</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Extend duplicate detection to payments + expenses/assets</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Audit finding (2026-08-25): duplicate detection covers ONLY invoices (_find_duplicate_invoice). Duplicate PAYMENTS and duplicate expenses/assets can also double-enter the books -- same money-correctness risk. Reuse the _dup_reason pattern (normalized ref + amount+party+date window) for payments/expenses so re-uploads are caught for every money record.</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>E3-06.2</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Surfaced in the founder-requested S6/S7 completeness audit.</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Epic 3 S6</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>E3-06.6</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>services/ingestion.py + validation</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>6</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Document AI</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Confidence calibration + review-routing for document/vision extraction</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Audit finding (2026-08-25): ai_extract_document returns the raw model confidence (0.7 default) with NO calibration or needs_review flag -- unlike ai_extract after E3-02.2. Extend the calibrate_confidence + needs_review pattern to the vision extractors (and optionally schema-validate + repair the OCR records like E3-02.1) so a shaky OCR extraction is flagged for review instead of looking identical to a confident one.</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>E3-02.1, E3-02.2</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Surfaced in the founder-requested S6/S7 completeness audit.</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Epic 3 S6</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>E3-06.7</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>routers/ledger.py (_num)</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>6</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Document AI</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Amount / currency normalization (lakh/crore/₹/commas)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Audit finding (2026-08-25, minor): _num() is a plain float() -- it does not parse Indian amount strings like "2.5 lakh", "₹1,20,000", or comma/word formats; it relies on the model emitting clean numbers. Add a tolerant amount parser for the India market so OCR/text amounts in local notation are captured correctly.</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Surfaced in the founder-requested S6/S7 completeness audit.</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Epic 3 S6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Epic 3 S6 (E3-06.5 DONE): duplicate detection for payments (double-entry parity)
Duplicate detection covered only invoices; a payment re-recorded twice is the same
double-entry risk. Added _find_duplicate_payment + pure _payment_dup_reason,
mirroring the invoice logic: a transaction reference (UTR/cheque/txn id -- globally
unique) is the strongest signal, then same invoice_number+amount, then amount+party
within the date window (a re-upload, NOT a recurring EMI/subscription). New
_find_duplicate_record checks invoices AND payments, and the WhatsApp capture flow
now calls it. Expenses/assets are covered transitively -- deduping the purchase
bill/invoice already prevents the double expense.

6 payment unit tests (recurring-EMI + cross-party false-positive traps). Exit gate +
fingerprint (260) hold.

Trackers side-by-side: Epic 3 Sprint 6 -> 5/7; Master Epic 3 -> 15/40. Dashboard regenerated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic3_AI_Foundation.xlsx
+++ b/docs/DecisionOS_Epic3_AI_Foundation.xlsx
@@ -1149,14 +1149,14 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D11" t="n">
         <v>7</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>57%</t>
+          <t>71%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -3645,7 +3645,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -3655,7 +3655,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Surfaced in the founder-requested S6/S7 completeness audit.</t>
+          <t>DONE. _find_duplicate_payment + pure _payment_dup_reason(pay,cand) mirror the invoice dedup for money records: reference (UTR/cheque/txn -- globally unique -&gt; strongest) &gt; same invoice_number+amount &gt; amount+party within INVOICE_DUP_WINDOW_DAYS (a re-upload, NOT a recurring EMI/subscription). New _find_duplicate_record(tenant,records) checks invoices AND payments; whatsapp capture flow now calls it (was invoice-only). Expenses/assets are covered transitively -- deduping the purchase bill/invoice prevents the double expense. 6 payment unit tests added (recurring-EMI + cross-party false-positive traps covered). Fingerprint 260.</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -3768,7 +3768,6 @@
           <t>Backlog</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
           <t>Surfaced in the founder-requested S6/S7 completeness audit.</t>

</xml_diff>